<commit_message>
updated figures and supplemental tables
</commit_message>
<xml_diff>
--- a/figures/Supplemental_Tables.xlsx
+++ b/figures/Supplemental_Tables.xlsx
@@ -1753,7 +1753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -1872,49 +1872,49 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.7160476190476192</v>
+        <v>0.7112380952380952</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1090153397154403</v>
+        <v>0.0965528544565291</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6710482984808017</v>
+        <v>0.6713830357513132</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7610469396144366</v>
+        <v>0.7510931547248773</v>
       </c>
       <c r="H3" t="n">
-        <v>5.874065289226414e-10</v>
+        <v>8.282546263761933e-11</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7790460273853129</v>
+        <v>0.7708087309515881</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1059440618891452</v>
+        <v>0.1023804259527414</v>
       </c>
       <c r="K3" t="n">
-        <v>0.6072380952380952</v>
+        <v>0.578</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1176389474522446</v>
+        <v>0.08375239727618961</v>
       </c>
       <c r="M3" t="n">
-        <v>0.7440369135508454</v>
+        <v>0.7138914896592914</v>
       </c>
       <c r="N3" t="n">
-        <v>0.8771428571428572</v>
+        <v>0.84</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3373333333333333</v>
+        <v>0.316</v>
       </c>
       <c r="P3" t="n">
-        <v>2055.68</v>
+        <v>2045.6</v>
       </c>
       <c r="Q3" t="n">
         <v>25</v>
       </c>
       <c r="R3" t="n">
-        <v>3.707613243436907e-09</v>
+        <v>8.282546263761933e-10</v>
       </c>
     </row>
     <row r="4">
@@ -1934,49 +1934,49 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.6987142857142858</v>
+        <v>0.7045238095238094</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1005305981857252</v>
+        <v>0.1058168608960151</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6572172943152613</v>
+        <v>0.6608447561239539</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7402112771133104</v>
+        <v>0.748202862923665</v>
       </c>
       <c r="H4" t="n">
-        <v>6.179355405728177e-10</v>
+        <v>9.540463145175875e-10</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7773232184482184</v>
+        <v>0.761744130869131</v>
       </c>
       <c r="J4" t="n">
-        <v>0.09883456973067296</v>
+        <v>0.1073181752288562</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6010238095238094</v>
+        <v>0.6056904761904761</v>
       </c>
       <c r="L4" t="n">
-        <v>0.09414701147388238</v>
+        <v>0.0974855843365528</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7336530232753142</v>
+        <v>0.7492629840060181</v>
       </c>
       <c r="N4" t="n">
-        <v>0.8607142857142859</v>
+        <v>0.9007142857142857</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3413333333333333</v>
+        <v>0.3106666666666667</v>
       </c>
       <c r="P4" t="n">
-        <v>2975.36</v>
+        <v>2969.84</v>
       </c>
       <c r="Q4" t="n">
         <v>25</v>
       </c>
       <c r="R4" t="n">
-        <v>3.707613243436907e-09</v>
+        <v>4.770231572587938e-09</v>
       </c>
     </row>
     <row r="5">
@@ -1996,49 +1996,49 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.6707619047619048</v>
+        <v>0.6516190476190477</v>
       </c>
       <c r="E5" t="n">
-        <v>0.09973100157792944</v>
+        <v>0.1065503236333157</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6295949706206226</v>
+        <v>0.6076372356814875</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7119288389031869</v>
+        <v>0.6956008595566078</v>
       </c>
       <c r="H5" t="n">
-        <v>9.312475211662744e-09</v>
+        <v>2.355627574022244e-07</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7576855862391576</v>
+        <v>0.7430394109858395</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0908804121371154</v>
+        <v>0.0963842173756624</v>
       </c>
       <c r="K5" t="n">
-        <v>0.619595238095238</v>
+        <v>0.6327380952380952</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1109940727837379</v>
+        <v>0.0889095913745956</v>
       </c>
       <c r="M5" t="n">
-        <v>0.6667638831756478</v>
+        <v>0.6726080586080586</v>
       </c>
       <c r="N5" t="n">
-        <v>0.6578571428571429</v>
+        <v>0.6521428571428571</v>
       </c>
       <c r="O5" t="n">
-        <v>0.5813333333333334</v>
+        <v>0.6133333333333334</v>
       </c>
       <c r="P5" t="n">
-        <v>2055.68</v>
+        <v>2045.6</v>
       </c>
       <c r="Q5" t="n">
         <v>25</v>
       </c>
       <c r="R5" t="n">
-        <v>3.724990084665098e-08</v>
+        <v>7.852091913407479e-07</v>
       </c>
     </row>
     <row r="6">
@@ -2058,40 +2058,40 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.6576666666666666</v>
+        <v>0.6414285714285713</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1648430132272101</v>
+        <v>0.1544471769281437</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5896228150878531</v>
+        <v>0.5776759101666705</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7257105182454802</v>
+        <v>0.7051812326904722</v>
       </c>
       <c r="H6" t="n">
-        <v>7.222857894175792e-05</v>
+        <v>0.0001212810302541</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7483505324041038</v>
+        <v>0.734195152070152</v>
       </c>
       <c r="J6" t="n">
-        <v>0.120915651253682</v>
+        <v>0.1205203663698666</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6307857142857142</v>
+        <v>0.5983095238095238</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1403050519611468</v>
+        <v>0.1054885905409487</v>
       </c>
       <c r="M6" t="n">
-        <v>0.631764020293432</v>
+        <v>0.6292874445815623</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5935714285714285</v>
+        <v>0.6392857142857143</v>
       </c>
       <c r="O6" t="n">
-        <v>0.6680000000000001</v>
+        <v>0.5573333333333332</v>
       </c>
       <c r="P6" t="n">
         <v>3</v>
@@ -2100,80 +2100,80 @@
         <v>25</v>
       </c>
       <c r="R6" t="n">
-        <v>0.000173348589460219</v>
+        <v>0.0003032025756353</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>single_omics</t>
+          <t>late_fusion_stacking</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>rna_all</t>
+          <t>rna_cnv_mutation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>stack_logistic_l2</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.6570714285714285</v>
+        <v>0.6138571428571428</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1386670904733625</v>
+        <v>0.1271600406020929</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5998324668568055</v>
+        <v>0.5613680578780987</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7143103902860516</v>
+        <v>0.6663462278361868</v>
       </c>
       <c r="H7" t="n">
-        <v>7.834422547427742e-06</v>
+        <v>0.0001570649451387</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7429206150991865</v>
+        <v>0.724613937649652</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1141546375588973</v>
+        <v>0.1091387331778859</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5965238095238096</v>
+        <v>0.584404761904762</v>
       </c>
       <c r="L7" t="n">
-        <v>0.09759616093500656</v>
+        <v>0.130796601968651</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7330479139024031</v>
+        <v>0.6145750915750916</v>
       </c>
       <c r="N7" t="n">
-        <v>0.8557142857142859</v>
+        <v>0.5821428571428572</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3373333333333333</v>
+        <v>0.5866666666666667</v>
       </c>
       <c r="P7" t="n">
-        <v>2055</v>
+        <v>3</v>
       </c>
       <c r="Q7" t="n">
         <v>25</v>
       </c>
       <c r="R7" t="n">
-        <v>2.350326764228323e-05</v>
+        <v>0.0003141298902775</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>single_omics</t>
+          <t>early_fusion</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rna_all</t>
+          <t>rna_cnv_mutation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2182,173 +2182,173 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.6182857142857143</v>
+        <v>0.6091904761904761</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1619784678459745</v>
+        <v>0.161973870638024</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5514242889253108</v>
+        <v>0.5423309484642479</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6851471396461178</v>
+        <v>0.6760500039167042</v>
       </c>
       <c r="H8" t="n">
-        <v>0.001265227019828171</v>
+        <v>0.0025339576996199</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7254346348096348</v>
+        <v>0.7035075935968793</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1246261373442671</v>
+        <v>0.1211582273141272</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5880000000000001</v>
+        <v>0.6441428571428571</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1322433301717161</v>
+        <v>0.124193434277082</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6196639841067085</v>
+        <v>0.695338831103537</v>
       </c>
       <c r="N8" t="n">
-        <v>0.6</v>
+        <v>0.7042857142857143</v>
       </c>
       <c r="O8" t="n">
-        <v>0.5760000000000001</v>
+        <v>0.5840000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>2055</v>
+        <v>2969.84</v>
       </c>
       <c r="Q8" t="n">
         <v>25</v>
       </c>
       <c r="R8" t="n">
-        <v>0.001897840529742256</v>
+        <v>0.0036199395708857</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>late_fusion_stacking</t>
+          <t>single_omics</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>rna_cnv_mutation</t>
+          <t>cnv</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>stack_logistic_l2</t>
+          <t>logistic_l2</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.612047619047619</v>
+        <v>0.4824285714285714</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1203732346016572</v>
+        <v>0.1548703374716134</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5623599898970444</v>
+        <v>0.4185012380792696</v>
       </c>
       <c r="G9" t="n">
-        <v>0.6617352481981935</v>
+        <v>0.5463559047778732</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0001000524602638307</v>
+        <v>0.5757823461393607</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7364384841349128</v>
+        <v>0.6442316631780918</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1083448764190559</v>
+        <v>0.0999520013869488</v>
       </c>
       <c r="K9" t="n">
-        <v>0.559595238095238</v>
+        <v>0.477047619047619</v>
       </c>
       <c r="L9" t="n">
-        <v>0.119447161876487</v>
+        <v>0.1284281747129137</v>
       </c>
       <c r="M9" t="n">
-        <v>0.6199362598186127</v>
+        <v>0.5538311427134956</v>
       </c>
       <c r="N9" t="n">
-        <v>0.6178571428571429</v>
+        <v>0.5714285714285715</v>
       </c>
       <c r="O9" t="n">
-        <v>0.5013333333333334</v>
+        <v>0.3826666666666666</v>
       </c>
       <c r="P9" t="n">
-        <v>3</v>
+        <v>539.24</v>
       </c>
       <c r="Q9" t="n">
         <v>25</v>
       </c>
       <c r="R9" t="n">
-        <v>0.0002001049205276614</v>
+        <v>0.5757823461393607</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>early_fusion</t>
+          <t>single_omics</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>rna_cnv_mutation</t>
+          <t>cnv</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>logistic_l2</t>
+          <t>random_forest</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.5884761904761905</v>
+        <v>0.4492380952380952</v>
       </c>
       <c r="E10" t="n">
-        <v>0.134739485066475</v>
+        <v>0.1587072949803183</v>
       </c>
       <c r="F10" t="n">
-        <v>0.5328584645915508</v>
+        <v>0.3837269436721446</v>
       </c>
       <c r="G10" t="n">
-        <v>0.6440939163608301</v>
+        <v>0.5147492468040458</v>
       </c>
       <c r="H10" t="n">
-        <v>0.003137624422548712</v>
+        <v>0.1228527339351806</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6963002969252969</v>
+        <v>0.6173872615479759</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1003625113503356</v>
+        <v>0.1051779081037125</v>
       </c>
       <c r="K10" t="n">
-        <v>0.609642857142857</v>
+        <v>0.5131428571428571</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1186908095313018</v>
+        <v>0.107694501396967</v>
       </c>
       <c r="M10" t="n">
-        <v>0.6583592757431767</v>
+        <v>0.649916110033757</v>
       </c>
       <c r="N10" t="n">
-        <v>0.6592857142857143</v>
+        <v>0.7342857142857143</v>
       </c>
       <c r="O10" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.292</v>
       </c>
       <c r="P10" t="n">
-        <v>2975.36</v>
+        <v>539.24</v>
       </c>
       <c r="Q10" t="n">
         <v>25</v>
       </c>
       <c r="R10" t="n">
-        <v>0.00418349923006495</v>
+        <v>0.1365030377057563</v>
       </c>
     </row>
     <row r="11">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>cnv</t>
+          <t>mutation</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2368,49 +2368,49 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.5272857142857142</v>
+        <v>0.4102380952380952</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1363185863764937</v>
+        <v>0.1835039661515479</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4710161674165922</v>
+        <v>0.3344913808794518</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5835552611548364</v>
+        <v>0.4859848095967386</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3269045751690324</v>
+        <v>0.0221639422836468</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6836615745365746</v>
+        <v>0.582289194932052</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1102727607687078</v>
+        <v>0.1009008709894832</v>
       </c>
       <c r="K11" t="n">
-        <v>0.5080238095238095</v>
+        <v>0.4573571428571428</v>
       </c>
       <c r="L11" t="n">
-        <v>0.103236796349748</v>
+        <v>0.09163394850033831</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6266260220687465</v>
+        <v>0.6494595311808934</v>
       </c>
       <c r="N11" t="n">
-        <v>0.6907142857142857</v>
+        <v>0.7907142857142858</v>
       </c>
       <c r="O11" t="n">
-        <v>0.3253333333333333</v>
+        <v>0.124</v>
       </c>
       <c r="P11" t="n">
-        <v>492.12</v>
+        <v>385</v>
       </c>
       <c r="Q11" t="n">
         <v>25</v>
       </c>
       <c r="R11" t="n">
-        <v>0.3566231729116717</v>
+        <v>0.0277049278545585</v>
       </c>
     </row>
     <row r="12">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>cnv</t>
+          <t>mutation</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2430,173 +2430,49 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.5101904761904762</v>
+        <v>0.359095238095238</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1236554100346564</v>
+        <v>0.1737500169932073</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4591480316088661</v>
+        <v>0.287374756064213</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5612329207720863</v>
+        <v>0.430815720126263</v>
       </c>
       <c r="H12" t="n">
-        <v>0.6839589593086419</v>
+        <v>0.0004587136820033</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6655256885971171</v>
+        <v>0.5448903536939251</v>
       </c>
       <c r="J12" t="n">
-        <v>0.09433680275755882</v>
+        <v>0.08245377401770281</v>
       </c>
       <c r="K12" t="n">
-        <v>0.4981904761904762</v>
+        <v>0.4362142857142857</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1016338152287868</v>
+        <v>0.1359017649987695</v>
       </c>
       <c r="M12" t="n">
-        <v>0.5561498501498501</v>
+        <v>0.5102813265166207</v>
       </c>
       <c r="N12" t="n">
-        <v>0.5457142857142857</v>
+        <v>0.5164285714285715</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4506666666666667</v>
+        <v>0.356</v>
       </c>
       <c r="P12" t="n">
-        <v>492.12</v>
+        <v>385</v>
       </c>
       <c r="Q12" t="n">
         <v>25</v>
       </c>
       <c r="R12" t="n">
-        <v>0.6839589593086419</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>single_omics</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>mutation</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>random_forest</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>0.4182857142857143</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.1486029836504336</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.3569454174437618</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.4796260111276668</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.01116286352393127</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.57839732291518</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.09279663110832968</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.4591428571428572</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.1126539374710888</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.6269816169382733</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.7342857142857143</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.184</v>
-      </c>
-      <c r="P13" t="n">
-        <v>427.56</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>25</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0.01339543622871753</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>single_omics</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>mutation</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>logistic_l2</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>0.3744761904761905</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.1573340437500776</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.3095318891580094</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.4394204917943716</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.0005416388307311614</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.5539650547864834</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0.08325041939911856</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0.4526666666666667</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.1325816440443041</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.5117090948267419</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0.4999999999999999</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0.4053333333333334</v>
-      </c>
-      <c r="P14" t="n">
-        <v>427.56</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>25</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0.000928523709824848</v>
+        <v>0.0007645228033389</v>
       </c>
     </row>
   </sheetData>
@@ -2610,7 +2486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -2715,15 +2591,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Proliferation (E2F/G2M/Mitotic Spindle/Myc)</t>
+          <t>Proliferation (E2F/G2M)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.090159189072188</v>
+        <v>1.81353544463483</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.45 to 2.53</t>
+          <t>1.72 to 1.90</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2732,7 +2608,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.0223837433328601</v>
+        <v>0.0017543225785731</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2751,16 +2627,16 @@
         <v>1.51661777556957</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9778023598690927</v>
+        <v>0.9778023598690928</v>
       </c>
       <c r="K3" t="n">
         <v>2.35234600730717</v>
       </c>
       <c r="L3" t="n">
-        <v>0.06292404768384986</v>
+        <v>0.06292404768384979</v>
       </c>
       <c r="M3" t="n">
-        <v>0.517</v>
+        <v>0.475</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -2768,17 +2644,13 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0.0943860715257748</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+        <v>0.1258480953676997</v>
+      </c>
+      <c r="P3" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="b">
+        <v>1</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -2789,11 +2661,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Interferon Gamma Response</t>
+          <t>Interferon Alpha Response</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-2.329968688733192</v>
+        <v>-3.849261455397972</v>
+      </c>
+      <c r="C4" t="n">
+        <v/>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2805,31 +2680,31 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>STAT1_sig</t>
+          <t>Module3_IFN_score</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>STAT1_sig</t>
+          <t>Module3_IFN_score</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>179</v>
       </c>
       <c r="I4" t="n">
-        <v>1.729839567436136</v>
+        <v>1.021531530354215</v>
       </c>
       <c r="J4" t="n">
-        <v>1.132791504014292</v>
+        <v>0.6902725522498652</v>
       </c>
       <c r="K4" t="n">
-        <v>2.641567242041996</v>
+        <v>1.51176033887856</v>
       </c>
       <c r="L4" t="n">
-        <v>0.01117364943075233</v>
+        <v>0.9151692129128844</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3</v>
+        <v>0.458</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -2837,88 +2712,15 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>0.03352094829225701</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
+        <v>0.9151692129128844</v>
+      </c>
+      <c r="P4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>0</v>
       </c>
       <c r="R4" t="inlineStr">
-        <is>
-          <t>discordant (significant)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Interferon Alpha Response</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-2.932767362763196</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Resistant</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Module3_IFN_score</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Module3_IFN_score</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>179</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1.021531530354215</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.6902725522498652</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1.51176033887856</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.9151692129128843</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Sensitive</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>0.9151692129128843</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
         <is>
           <t>null / inconclusive</t>
         </is>
@@ -5008,7 +4810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="22.5" customWidth="1" min="1" max="1"/>
@@ -5059,13 +4861,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-2.951381236364488</v>
+        <v>-2.972876944569204</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>-2.45610135813259</v>
+        <v>-2.476837866713567</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -5078,13 +4880,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-2.942198128759167</v>
+        <v>-2.912554422685802</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>-2.422317602697819</v>
+        <v>-2.442720055269889</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -5097,13 +4899,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-2.29402564743974</v>
+        <v>-2.272731914736729</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>-2.641682919838547</v>
+        <v>-2.698372314432666</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -5116,16 +4918,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-2.001375290488051</v>
+        <v>-1.992642012726588</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0005775339301183</v>
+        <v>0.0002961792871951</v>
       </c>
       <c r="D6" t="n">
-        <v>-1.907338859616113</v>
+        <v>-1.883157578809065</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0002545757336289</v>
+        <v>0.0005378348253613</v>
       </c>
     </row>
     <row r="7">
@@ -5135,35 +4937,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-1.663709525631336</v>
+        <v>-1.667012760015685</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0077704565143202</v>
+        <v>0.0077545122465647</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.911637252022791</v>
+        <v>-1.84618694712538</v>
       </c>
       <c r="E7" t="n">
-        <v>0.000297005022567</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Unfolded Protein Response</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>-1.543757575791826</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.0182244040170693</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-1.458721266433515</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.0486098220268117</v>
+        <v>0.0007376020462097999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>